<commit_message>
fix: bizfit_stop Pcode 필수화 + 메모 기능 제거
kimpro reception.html 강제종료 모달과 동일 정책으로 통일(같은 백엔드 공유).
pcode 없는 MID-only 입력은 더 이상 처리하지 않음, 메모 입력/표시 삭제.
</commit_message>
<xml_diff>
--- a/macro/양식/임시중단_강제종료_양식.xlsx
+++ b/macro/양식/임시중단_강제종료_양식.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -478,11 +478,6 @@
           <t>강제종료</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>메모</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -490,7 +485,11 @@
           <t>1839711962</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>P2116A864DC2B0CF2</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>O</t>
@@ -499,11 +498,6 @@
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>O</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>예: MID 전체 캠페인 임시중단</t>
         </is>
       </c>
     </row>

</xml_diff>